<commit_message>
Remocao da IA do bot
</commit_message>
<xml_diff>
--- a/banco_de_dados.xlsx
+++ b/banco_de_dados.xlsx
@@ -499,7 +499,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1230,9 +1230,156 @@
         <v>Concluído</v>
       </c>
     </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26">
+        <v>29</v>
+      </c>
+      <c r="B26" t="str">
+        <v>22/04/2026, 16:52:06</v>
+      </c>
+      <c r="C26" t="str">
+        <v>22/04/2026, 16:56:10</v>
+      </c>
+      <c r="D26" t="str">
+        <v>22/04/2026, 16:56:17</v>
+      </c>
+      <c r="E26" t="str">
+        <v>8057895547051@lid</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Lucas Barba Santos</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Programas | ERP</v>
+      </c>
+      <c r="H26" t="str" xml:space="preserve">
+        <v xml:space="preserve">AOKI perdeu conexão, não consegue estabilizar.
+Saí e tentei logar novamente, porém só fica carregando e não dá nenhum outro sinal.
+Já verifiquei a conexão do notebook e está tudo em ordem.</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Concluído</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>30</v>
+      </c>
+      <c r="B27" t="str">
+        <v>24/04/2026, 10:22:03</v>
+      </c>
+      <c r="C27" t="str">
+        <v>24/04/2026, 11:52:38</v>
+      </c>
+      <c r="D27" t="str">
+        <v>27/04/2026, 07:34:09</v>
+      </c>
+      <c r="E27" t="str">
+        <v>8057895547051@lid</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Lucas Barba Santos</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Impressora | Scanner</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Impressora demora mais de 15 minutos para imprimir um documento que foi solicitado.</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Concluído</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>31</v>
+      </c>
+      <c r="B28" t="str">
+        <v>27/04/2026, 14:36:31</v>
+      </c>
+      <c r="C28" t="str">
+        <v>27/04/2026, 15:22:37</v>
+      </c>
+      <c r="D28" t="str">
+        <v>27/04/2026, 15:26:43</v>
+      </c>
+      <c r="E28" t="str">
+        <v>8057895547051@lid</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Lucas Barba Santos</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Acesso | Contas</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Necessito do acesso ao drive no notebook, por favor</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Concluído</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>32</v>
+      </c>
+      <c r="B29" t="str">
+        <v>28/04/2026, 12:40:24</v>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v>28/04/2026, 12:43:05</v>
+      </c>
+      <c r="E29" t="str">
+        <v>55933761798339@lid</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Diego Redekop Guidem</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Internet</v>
+      </c>
+      <c r="H29" t="str">
+        <v>meu pc nao liga</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Concluído</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>33</v>
+      </c>
+      <c r="B30" t="str">
+        <v>28/04/2026, 14:24:41</v>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v>28/04/2026, 14:24:56</v>
+      </c>
+      <c r="E30" t="str">
+        <v>55933761798339@lid</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Diego Redekop Guidem</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Outros</v>
+      </c>
+      <c r="H30" t="str">
+        <v>minha internet nao funciona</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Concluído</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>